<commit_message>
n8n board refresh 2026-10-20T17:42:25Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-20 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>157.82</v>
+        <v>161.87</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>73.63</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.143</v>
+        <v>1.163</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05245999813079834</v>
+        <v>0.05126999855041504</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284967.323102</v>
+        <v>120284977.4215097</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>73.63</v>
+        <v>74.84999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8856582144</v>
+        <v>9003330560</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.58</v>
+        <v>11.77</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.869999999999999</v>
+        <v>9.98</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1141196928</v>
+        <v>1040550976</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-12.08</v>
+        <v>-10.069</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>6.564</v>
+        <v>5.471</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>13403847680</v>
+        <v>13453901824</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>25.104305</v>
+        <v>25.198053</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.507</v>
+        <v>15.824</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.927</v>
+        <v>1.967</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>3773949952</v>
+        <v>4135661824</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>16.467468</v>
+        <v>18.045782</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>11.133</v>
+        <v>11.602</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.243</v>
+        <v>1.295</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1581667200</v>
+        <v>1794110464</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>14.308595</v>
+        <v>16.230469</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.106</v>
+        <v>5.445</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>43520942080</v>
+        <v>51176091648</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>13.265432</v>
+        <v>15.598765</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>18.857</v>
+        <v>21.567</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.164</v>
+        <v>4.762</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2102499200</v>
+        <v>1897922432</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>47.403103</v>
+        <v>42.7907</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>31.352</v>
+        <v>27.174</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.857</v>
+        <v>5.076</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>15269892096</v>
+        <v>16016570368</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>11.361344</v>
+        <v>11.9169</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>8.75</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.182</v>
+        <v>1.231</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>5642982912</v>
+        <v>5643192832</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>15.71587</v>
+        <v>15.716454</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>10.642</v>
+        <v>10.832</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.083</v>
+        <v>1.102</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-21T17:41:26Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-20 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-21 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>161.87</v>
+        <v>162.6</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>74.84999999999999</v>
+        <v>74.58499999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.163</v>
+        <v>1.18</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05126999855041504</v>
+        <v>0.05105999946594238</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284977.4215097</v>
+        <v>120284969.6855936</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>74.84999999999999</v>
+        <v>74.58499999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9003330560</v>
+        <v>8971454464</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.77</v>
+        <v>11.73</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>9.98</v>
+        <v>10.07</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1040550976</v>
+        <v>1059682880</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.069</v>
+        <v>-10.404</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.471</v>
+        <v>5.653</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>13453901824</v>
+        <v>13696224256</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>25.198053</v>
+        <v>25.651905</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.824</v>
+        <v>15.662</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.967</v>
+        <v>1.946</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4135661824</v>
+        <v>4089826560</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>18.045782</v>
+        <v>17.845781</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>11.602</v>
+        <v>11.761</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.295</v>
+        <v>1.313</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1794110464</v>
+        <v>1839233280</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>16.230469</v>
+        <v>16.638672</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.445</v>
+        <v>5.61</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.869</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>51176091648</v>
+        <v>51358580736</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>15.598765</v>
+        <v>15.654322</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>21.567</v>
+        <v>22.399</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.762</v>
+        <v>4.946</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1897922432</v>
+        <v>2061240064</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>42.7907</v>
+        <v>46.47287</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>27.174</v>
+        <v>27.78</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.076</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>16016570368</v>
+        <v>16110062592</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>11.9169</v>
+        <v>11.986462</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.109999999999999</v>
+        <v>9.195</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.231</v>
+        <v>1.242</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>5643192832</v>
+        <v>5733691904</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>15.716454</v>
+        <v>15.968496</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>10.832</v>
+        <v>10.942</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.102</v>
+        <v>1.113</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-22T17:41:33Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-21 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-22 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>162.6</v>
+        <v>167.73</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>74.58499999999999</v>
+        <v>78.67</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.18</v>
+        <v>1.132</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05105999946594238</v>
+        <v>0.04963000297546387</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284969.6855936</v>
+        <v>120284972.8740308</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>74.58499999999999</v>
+        <v>78.67</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8971454464</v>
+        <v>9462818816</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>11.73</v>
+        <v>12.37</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.07</v>
+        <v>10.08</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.14</v>
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1059682880</v>
+        <v>1016528256</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.404</v>
+        <v>-10.538</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.653</v>
+        <v>5.726</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>13696224256</v>
+        <v>13599539200</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>25.651905</v>
+        <v>25.2617</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.662</v>
+        <v>15.953</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.946</v>
+        <v>1.982</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4089826560</v>
+        <v>4314446848</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>17.845781</v>
+        <v>18.825903</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>11.761</v>
+        <v>11.681</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.313</v>
+        <v>1.304</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1839233280</v>
+        <v>1919331328</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>16.638672</v>
+        <v>17.363281</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.61</v>
+        <v>5.78</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.895</v>
+        <v>0.922</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>51358580736</v>
+        <v>52836962304</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>15.654322</v>
+        <v>16.104939</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>22.399</v>
+        <v>22.561</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.946</v>
+        <v>4.982</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2061240064</v>
+        <v>2018949376</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>46.47287</v>
+        <v>45.519382</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>27.78</v>
+        <v>30.98</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.19</v>
+        <v>5.788</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>16110062592</v>
+        <v>16708032512</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>11.986462</v>
+        <v>12.431373</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.195</v>
+        <v>9.278</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.242</v>
+        <v>1.253</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>5733691904</v>
+        <v>5915107840</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>15.968496</v>
+        <v>16.473745</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>10.942</v>
+        <v>11.033</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.113</v>
+        <v>1.122</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-23T17:42:13Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-22 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-23 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>167.73</v>
+        <v>166.67</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>78.67</v>
+        <v>78.22499999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.132</v>
+        <v>1.131</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04963000297546387</v>
+        <v>0.04991999626159668</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284972.8740308</v>
+        <v>120284976.5164589</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>78.67</v>
+        <v>78.22499999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9462818816</v>
+        <v>9409292288</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>12.37</v>
+        <v>12.3</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.08</v>
+        <v>10.41</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.14</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1016528256</v>
+        <v>1018925824</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.538</v>
+        <v>-10.136</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.726</v>
+        <v>5.507</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>13599539200</v>
+        <v>14035452928</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>25.2617</v>
+        <v>26.071426</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.953</v>
+        <v>14.96</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.982</v>
+        <v>1.916</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4314446848</v>
+        <v>4302711808</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>18.825903</v>
+        <v>18.774698</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>11.681</v>
+        <v>12.188</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.304</v>
+        <v>1.361</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1919331328</v>
+        <v>1958624640</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>17.363281</v>
+        <v>17.71875</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.78</v>
+        <v>6.063</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.922</v>
+        <v>0.968</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>52836962304</v>
+        <v>50589007872</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>16.104939</v>
+        <v>15.419753</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>22.561</v>
+        <v>23.411</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.982</v>
+        <v>5.169</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2018949376</v>
+        <v>2059176960</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>45.519382</v>
+        <v>46.426357</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>30.98</v>
+        <v>30.476</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.788</v>
+        <v>5.693</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>16708032512</v>
+        <v>17099567104</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>12.431373</v>
+        <v>12.722689</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.278</v>
+        <v>9.567</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.253</v>
+        <v>1.292</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>5915107840</v>
+        <v>6107837440</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>16.473745</v>
+        <v>17.010502</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>11.033</v>
+        <v>11.411</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.122</v>
+        <v>1.161</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-24T17:40:51Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-23 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-24 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>166.67</v>
+        <v>127.87</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>78.22499999999999</v>
+        <v>78.31999999999999</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>1.131</v>
+        <v>0.633</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04991999626159668</v>
+        <v>0.0498799991607666</v>
       </c>
     </row>
     <row r="6">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>4160000000</v>
+        <v>4707999744</v>
       </c>
     </row>
     <row r="33">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>540000000</v>
+        <v>334000000</v>
       </c>
     </row>
     <row r="34">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>120284976.5164589</v>
+        <v>119096965.8835547</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>78.22499999999999</v>
+        <v>78.31999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9409292288</v>
+        <v>9327674368</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>12.3</v>
+        <v>12.31</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>10.41</v>
+        <v>11.13</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.18</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1018925824</v>
+        <v>1026118272</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.136</v>
+        <v>-10.203</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.507</v>
+        <v>5.544</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>14035452928</v>
+        <v>14010701824</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>26.071426</v>
+        <v>26.02545</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>14.96</v>
+        <v>15.276</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.916</v>
+        <v>1.956</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4302711808</v>
+        <v>4341644288</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>18.774698</v>
+        <v>18.944578</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>12.188</v>
+        <v>12.166</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.361</v>
+        <v>1.358</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1958624640</v>
+        <v>1944375296</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>17.71875</v>
+        <v>17.589844</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>6.063</v>
+        <v>5.981</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.968</v>
+        <v>0.954</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>50589007872</v>
+        <v>50022150144</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>15.419753</v>
+        <v>15.246914</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>23.411</v>
+        <v>21.081</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>5.169</v>
+        <v>4.763</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2059176960</v>
+        <v>2041985664</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>46.426357</v>
+        <v>46.03876</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>30.476</v>
+        <v>30.301</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.693</v>
+        <v>5.661</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>17099567104</v>
+        <v>17076979712</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>12.722689</v>
+        <v>12.705882</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.567</v>
+        <v>9.638999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.292</v>
+        <v>1.302</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>6107837440</v>
+        <v>6105742336</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>17.010502</v>
+        <v>17.004667</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>11.411</v>
+        <v>11.534</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.161</v>
+        <v>1.173</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-25T17:41:05Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-24 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-25 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>127.87</v>
+        <v>162.15</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.633</v>
+        <v>1.07</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8">
@@ -1644,7 +1644,7 @@
         <v>15.246914</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>21.081</v>
+        <v>21.501</v>
       </c>
       <c r="F10" s="34" t="n">
         <v>4.763</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-10-27T17:41:10Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-26 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>162.37</v>
+        <v>161.97</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>84.11</v>
+        <v>83.04000000000001</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.93</v>
+        <v>0.951</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.0498199987411499</v>
+        <v>0.04993000030517578</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>119096970.7288075</v>
+        <v>119096971.0982659</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>84.11</v>
+        <v>83.04000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10017246208</v>
+        <v>9889812480</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.22</v>
+        <v>13.06</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>11.13</v>
+        <v>11.62</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.24</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="6">
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1032159872</v>
+        <v>1126812032</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.203</v>
+        <v>-10.069</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.544</v>
+        <v>5.471</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>14793800704</v>
+        <v>14605623296</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>27.48009</v>
+        <v>27.130543</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.276</v>
+        <v>15.828</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>1.956</v>
+        <v>2.027</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4446844416</v>
+        <v>4381681152</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>19.403614</v>
+        <v>19.119276</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>12.166</v>
+        <v>12.423</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.358</v>
+        <v>1.387</v>
       </c>
     </row>
     <row r="9">
@@ -1614,13 +1614,13 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1917604096</v>
+        <v>1838585600</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>17.347656</v>
+        <v>16.632814</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.981</v>
+        <v>5.978</v>
       </c>
       <c r="F9" s="34" t="n">
         <v>0.954</v>
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>49880383488</v>
+        <v>49009557504</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>15.203703</v>
+        <v>14.938272</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>21.501</v>
+        <v>21.645</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.763</v>
+        <v>4.795</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>2072070528</v>
+        <v>1515243520</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>46.717056</v>
+        <v>34.162792</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>30.301</v>
+        <v>30.603</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.661</v>
+        <v>5.717</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>17519339520</v>
+        <v>17517457408</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>13.035013</v>
+        <v>13.033613</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.638999999999999</v>
+        <v>9.837999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.302</v>
+        <v>1.329</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>6267886592</v>
+        <v>6222008832</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>17.456244</v>
+        <v>17.328472</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>11.534</v>
+        <v>11.688</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.173</v>
+        <v>1.189</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-28T17:41:21Z
</commit_message>
<xml_diff>
--- a/app/reports/BAH_research.xlsx
+++ b/app/reports/BAH_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-27 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-28 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>161.97</v>
+        <v>161.12</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>83.04000000000001</v>
+        <v>83.41</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.951</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04993000030517578</v>
+        <v>0.05015999794006348</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>119096971.0982659</v>
+        <v>119096970.0515526</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>83.04000000000001</v>
+        <v>83.41</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9889812480</v>
+        <v>9933878272</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.06</v>
+        <v>12.95</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>11.62</v>
+        <v>11.63</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.3</v>
@@ -1544,14 +1544,14 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>1126812032</v>
+        <v>1141196928</v>
       </c>
       <c r="D6" s="34" t="n"/>
       <c r="E6" s="34" t="n">
-        <v>-10.069</v>
+        <v>-11.611</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>5.471</v>
+        <v>6.309</v>
       </c>
     </row>
     <row r="7">
@@ -1566,16 +1566,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>14605623296</v>
+        <v>14608937984</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>27.130543</v>
+        <v>27.136698</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.828</v>
+        <v>15.85</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>2.027</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1590,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>4381681152</v>
+        <v>4389826560</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>19.119276</v>
+        <v>19.15482</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>12.423</v>
+        <v>12.263</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>1.387</v>
+        <v>1.369</v>
       </c>
     </row>
     <row r="9">
@@ -1614,16 +1614,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>1838585600</v>
+        <v>1876367744</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>16.632814</v>
+        <v>16.974611</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>5.978</v>
+        <v>5.755</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.954</v>
+        <v>0.918</v>
       </c>
     </row>
     <row r="10">
@@ -1638,16 +1638,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>49009557504</v>
+        <v>49191825408</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>14.938272</v>
+        <v>14.993828</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>21.645</v>
+        <v>21.07</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>4.795</v>
+        <v>4.668</v>
       </c>
     </row>
     <row r="11">
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>1515243520</v>
+        <v>1653117952</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>34.162792</v>
+        <v>37.27132</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>30.603</v>
+        <v>21.8</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.717</v>
+        <v>4.073</v>
       </c>
     </row>
     <row r="12">
@@ -1686,16 +1686,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>17517457408</v>
+        <v>17427101696</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>13.033613</v>
+        <v>12.966386</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.837999999999999</v>
+        <v>9.826000000000001</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>1.329</v>
+        <v>1.327</v>
       </c>
     </row>
     <row r="13">
@@ -1710,16 +1710,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>6222008832</v>
+        <v>6205040128</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>17.328472</v>
+        <v>17.281216</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>11.688</v>
+        <v>11.744</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>1.189</v>
+        <v>1.195</v>
       </c>
     </row>
     <row r="15">

</xml_diff>